<commit_message>
chore: user manual format and color changes for print footer
</commit_message>
<xml_diff>
--- a/out/calculadora-simples-nacional-configuracoes.xlsx
+++ b/out/calculadora-simples-nacional-configuracoes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thais Camilo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B997C989-C75F-483D-A185-910821A964D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F616698-BE15-483B-A9DC-18E6A222CD45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -145,31 +145,31 @@
     <t>REPARTICAO_ANEXO_I</t>
   </si>
   <si>
+    <t>33.5</t>
+  </si>
+  <si>
+    <t>Percentual destinado ao ICMS na 5ª Faixa do Anexo I (Comércio). Fonte: LC 155/2016, Anexo I.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REPARTICAO_ANEXO_II	</t>
+  </si>
+  <si>
+    <t>32.0</t>
+  </si>
+  <si>
+    <t>Percentual destinado ao ICMS na 5ª Faixa do Anexo II (Indústria). Fonte: LC 155/2016, Anexo II.</t>
+  </si>
+  <si>
+    <t>REPARTICAO_ANEXO_III</t>
+  </si>
+  <si>
+    <t>Percentual destinado ao ISS na 5ª Faixa do Anexo III (Serviços). Fonte: LC 155/2016, Anexo III.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REPARTICAO_ANEXO_IV	</t>
+  </si>
+  <si>
     <t>40.0</t>
-  </si>
-  <si>
-    <t>Percentual destinado ao ICMS na 5ª Faixa do Anexo I (Comércio). Fonte: LC 155/2016, Anexo I.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REPARTICAO_ANEXO_II	</t>
-  </si>
-  <si>
-    <t>32.0</t>
-  </si>
-  <si>
-    <t>Percentual destinado ao ICMS na 5ª Faixa do Anexo II (Indústria). Fonte: LC 155/2016, Anexo II.</t>
-  </si>
-  <si>
-    <t>REPARTICAO_ANEXO_III</t>
-  </si>
-  <si>
-    <t>33.5</t>
-  </si>
-  <si>
-    <t>Percentual destinado ao ISS na 5ª Faixa do Anexo III (Serviços). Fonte: LC 155/2016, Anexo III.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REPARTICAO_ANEXO_IV	</t>
   </si>
   <si>
     <t>Percentual destinado ao ISS na 5ª Faixa do Anexo IV (Serviços). Fonte: LC 155/2016, Anexo IV.</t>
@@ -1416,18 +1416,18 @@
         <v>40</v>
       </c>
       <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
         <v>41</v>
-      </c>
-      <c r="C6" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
         <v>43</v>
-      </c>
-      <c r="B7" t="s">
-        <v>35</v>
       </c>
       <c r="C7" t="s">
         <v>44</v>

</xml_diff>